<commit_message>
Included changes for Removing TP data for all countries.
</commit_message>
<xml_diff>
--- a/Data/Input/FiscalCalendar_2026_07/Fiscal_Calander.xlsx
+++ b/Data/Input/FiscalCalendar_2026_07/Fiscal_Calander.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aws-svc-rpa52d\Documents\UiPath\3043_LATAM_DataLoad\Data\Input\FiscalCalendar_2026_07\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{908E6737-4A91-41F8-AA09-65854F0E625B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D624403-C21E-4DED-ADEA-42E05E2FB264}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LATAM_2026" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="20">
   <si>
     <t>MonitoringStart_Date</t>
   </si>
@@ -82,6 +83,9 @@
   </si>
   <si>
     <t>InvoiceStatus</t>
+  </si>
+  <si>
+    <t>InProgress</t>
   </si>
 </sst>
 </file>
@@ -555,7 +559,7 @@
         <v>46203</v>
       </c>
       <c r="C7" s="3">
-        <v>46255</v>
+        <v>46205</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>15</v>
@@ -586,16 +590,16 @@
         <v>10</v>
       </c>
       <c r="B9" s="3">
-        <v>46266</v>
+        <v>46262</v>
       </c>
       <c r="C9" s="3">
-        <v>46268</v>
+        <v>46264</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -670,4 +674,242 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBC2E586-9BEA-4B86-8AB1-6FD8BFC564AD}">
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20.28515625" customWidth="1"/>
+    <col min="2" max="2" width="21" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" customWidth="1"/>
+    <col min="4" max="4" width="22.28515625" customWidth="1"/>
+    <col min="5" max="5" width="22.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="3">
+        <v>46056</v>
+      </c>
+      <c r="C2" s="3">
+        <v>46058</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="3">
+        <v>46084</v>
+      </c>
+      <c r="C3" s="3">
+        <v>46086</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="3">
+        <v>46112</v>
+      </c>
+      <c r="C4" s="3">
+        <v>46114</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="3">
+        <v>46147</v>
+      </c>
+      <c r="C5" s="3">
+        <v>46149</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="3">
+        <v>46175</v>
+      </c>
+      <c r="C6" s="3">
+        <v>46177</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="3">
+        <v>46203</v>
+      </c>
+      <c r="C7" s="3">
+        <v>46255</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="3">
+        <v>46238</v>
+      </c>
+      <c r="C8" s="3">
+        <v>46240</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="3">
+        <v>46266</v>
+      </c>
+      <c r="C9" s="3">
+        <v>46268</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="3">
+        <v>46294</v>
+      </c>
+      <c r="C10" s="3">
+        <v>46296</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="3">
+        <v>46329</v>
+      </c>
+      <c r="C11" s="3">
+        <v>46331</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="3">
+        <v>46357</v>
+      </c>
+      <c r="C12" s="3">
+        <v>46359</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="3">
+        <v>46392</v>
+      </c>
+      <c r="C13" s="3">
+        <v>46394</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>